<commit_message>
Align BOM scope labels and isolation-relay diagram with the published review.
Keep reused mower parts as reference rows, tap the isolation coil from the retract/disengage lead, and label the receiver as four channels used.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/02-components/bill-of-materials.xlsx
+++ b/02-components/bill-of-materials.xlsx
@@ -224,6 +224,12 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Front wheel mounting points</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Notes</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Existing/reused—reference only</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -508,6 +514,7 @@
     <x:col min="5" max="5" width="40" customWidth="1"/>
     <x:col min="6" max="6" width="31" customWidth="1"/>
     <x:col min="7" max="7" width="42" customWidth="1"/>
+    <x:col min="8" max="8" width="36" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
@@ -532,6 +539,9 @@
       <x:c r="G1" s="1" t="s">
         <x:v>6</x:v>
       </x:c>
+      <x:c r="H1" s="1" t="s">
+        <x:v>72</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="2" t="s">
@@ -555,6 +565,9 @@
       <x:c r="G2" s="2" t="s">
         <x:v>12</x:v>
       </x:c>
+      <x:c r="H2" s="3" t="s">
+        <x:v>73</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="2" t="s">
@@ -577,6 +590,9 @@
       </x:c>
       <x:c r="G3" s="2" t="s">
         <x:v>18</x:v>
+      </x:c>
+      <x:c r="H3" s="3" t="s">
+        <x:v>73</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="36" customHeight="1">

</xml_diff>

<commit_message>
Document the motor drivers and replace the original mower photos.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/02-components/bill-of-materials.xlsx
+++ b/02-components/bill-of-materials.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Re4773c9c8dc2412f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Re12c48e57339465e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -31,6 +31,9 @@
     <x:t xml:space="preserve">Reason for Selection</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">Notes</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">Base Platform</x:t>
   </x:si>
   <x:si>
@@ -49,6 +52,9 @@
     <x:t xml:space="preserve">Retains the original mower platform and existing safety systems</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">Existing/reused—reference only</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">Drive System</x:t>
   </x:si>
   <x:si>
@@ -226,10 +232,31 @@
     <x:t xml:space="preserve">Front wheel mounting points</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Notes</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Existing/reused—reference only</x:t>
+    <x:t xml:space="preserve">Small rollers mount around the original wheel to allow lateral rolling and reduce turning resistance</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">BLDC Motor Driver Board</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Jiqu Technology; sensorless RC version; 6-60 V DC; 600 W; 40 A peak; forward/reverse and braking; PWM/0-5 V/potentiometer speed control; overtemperature/overcurrent protection; 63 x 45 x 36 mm</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Controls speed and direction of a sensorless brushless DC motor</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">RC control, reversible operation and braking support remote motor control</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Brushed DC Motor Driver</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Jiqu Technology DC85V50-K RC version; listing advertises 800 W and 24/48/85 V; receiver connector; forward/reverse speed control; aluminum enclosure</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Controls speed and direction of a brushed DC motor</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Receiver connection and reversible speed control support remote operation of a brushed motor</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -284,7 +311,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="8">
+  <x:cellXfs count="9">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -305,6 +332,9 @@
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -540,82 +570,82 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="H1" s="1" t="s">
-        <x:v>72</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B2" s="2" t="s">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C2" s="2" t="s">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D2" s="4">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E2" s="2" t="s">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="F2" s="2" t="s">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G2" s="2" t="s">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="H2" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="2" t="s">
-        <x:v>13</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="B3" s="2" t="s">
-        <x:v>14</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C3" s="2" t="s">
-        <x:v>15</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="D3" s="4">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E3" s="2" t="s">
-        <x:v>16</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="F3" s="2" t="s">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="G3" s="2" t="s">
-        <x:v>18</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="H3" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="5" t="s">
-        <x:v>19</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="B4" s="5" t="s">
-        <x:v>20</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C4" s="5" t="s">
-        <x:v>21</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="D4" s="6">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E4" s="5" t="s">
-        <x:v>22</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="F4" s="5" t="s">
-        <x:v>23</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="G4" s="5" t="s">
-        <x:v>24</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="H4" s="7"/>
       <x:c r="I4" s="7"/>
@@ -1113,205 +1143,235 @@
     </x:row>
     <x:row r="5" ht="24" customHeight="1">
       <x:c r="A5" s="2" t="s">
-        <x:v>19</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="B5" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="C5" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="D5" s="4">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E5" s="2" t="s">
-        <x:v>27</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F5" s="2" t="s">
-        <x:v>28</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="G5" s="2" t="s">
-        <x:v>29</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="24" customHeight="1">
       <x:c r="A6" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="B6" s="2" t="s">
-        <x:v>31</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="C6" s="2" t="s">
-        <x:v>32</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="D6" s="4">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E6" s="2" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="F6" s="2" t="s">
-        <x:v>34</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="G6" s="2" t="s">
-        <x:v>35</x:v>
+        <x:v>37</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="24" customHeight="1">
       <x:c r="A7" s="2" t="s">
-        <x:v>36</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="B7" s="2" t="s">
-        <x:v>37</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="C7" s="2" t="s">
-        <x:v>38</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="D7" s="4">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E7" s="2" t="s">
-        <x:v>39</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="F7" s="2" t="s">
-        <x:v>28</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="G7" s="2" t="s">
-        <x:v>40</x:v>
+        <x:v>42</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="24" customHeight="1">
       <x:c r="A8" s="2" t="s">
-        <x:v>36</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="B8" s="2" t="s">
-        <x:v>41</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="C8" s="2" t="s">
-        <x:v>42</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="D8" s="4" t="s">
-        <x:v>43</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="E8" s="2" t="s">
-        <x:v>44</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="F8" s="2" t="s">
-        <x:v>28</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="G8" s="2" t="s">
-        <x:v>45</x:v>
+        <x:v>47</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
       <x:c r="A9" s="2" t="s">
-        <x:v>46</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="B9" s="2" t="s">
-        <x:v>47</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="C9" s="2" t="s">
-        <x:v>48</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="D9" s="4">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E9" s="2" t="s">
-        <x:v>49</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="F9" s="2" t="s">
-        <x:v>50</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="G9" s="2" t="s">
-        <x:v>51</x:v>
+        <x:v>53</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="24" customHeight="1">
       <x:c r="A10" s="2" t="s">
-        <x:v>52</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="B10" s="2" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C10" s="2" t="s">
-        <x:v>54</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="D10" s="4" t="s">
-        <x:v>55</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="E10" s="2" t="s">
-        <x:v>56</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="F10" s="2" t="s">
-        <x:v>57</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="G10" s="2" t="s">
-        <x:v>58</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="24" customHeight="1">
       <x:c r="A11" s="2" t="s">
-        <x:v>59</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="B11" s="2" t="s">
-        <x:v>60</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C11" s="2" t="s">
-        <x:v>61</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="D11" s="4" t="s">
-        <x:v>62</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="E11" s="2" t="s">
-        <x:v>63</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="F11" s="2" t="s">
-        <x:v>64</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="G11" s="2" t="s">
-        <x:v>65</x:v>
+        <x:v>67</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
       <x:c r="A12" s="3" t="s">
-        <x:v>66</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="B12" s="2" t="s">
-        <x:v>67</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="C12" s="2" t="s">
-        <x:v>68</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="D12" s="4" t="s">
-        <x:v>69</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="E12" s="2" t="s">
-        <x:v>70</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="F12" s="2" t="s">
-        <x:v>71</x:v>
-      </x:c>
-      <x:c r="G12" s="2" t="str">
-        <x:v>Small rollers mount around the original wheel to allow lateral rolling and reduce turning resistance</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="24" customHeight="1">
-      <x:c r="A13" s="2"/>
-      <x:c r="B13" s="2"/>
-      <x:c r="C13" s="2"/>
-      <x:c r="D13" s="4"/>
-      <x:c r="E13" s="2"/>
-      <x:c r="F13" s="2"/>
-      <x:c r="G13" s="2"/>
-    </x:row>
-    <x:row r="14" ht="24" customHeight="1">
-      <x:c r="A14" s="2"/>
-      <x:c r="B14" s="2"/>
-      <x:c r="C14" s="2"/>
-      <x:c r="D14" s="4"/>
-      <x:c r="E14" s="2"/>
-      <x:c r="F14" s="2"/>
-      <x:c r="G14" s="2"/>
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="G12" s="2" t="s">
+        <x:v>74</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="52.79999923706055" customHeight="1">
+      <x:c r="A13" s="2" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="B13" s="2" t="s">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="C13" s="2" t="s">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="D13" s="4">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E13" s="2" t="s">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="F13" s="2" t="str">
+        <x:v>Rear electronics enclosure, behind the rear axle</x:v>
+      </x:c>
+      <x:c r="G13" s="2" t="s">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="H13" s="8"/>
+    </x:row>
+    <x:row r="14" ht="66" customHeight="1">
+      <x:c r="A14" s="2" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="B14" s="2" t="s">
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="C14" s="2" t="s">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="D14" s="4">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E14" s="2" t="s">
+        <x:v>81</x:v>
+      </x:c>
+      <x:c r="F14" s="2" t="str">
+        <x:v>Rear electronics enclosure, behind the rear axle</x:v>
+      </x:c>
+      <x:c r="G14" s="2" t="s">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="H14" s="8"/>
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
       <x:c r="A15" s="2"/>

</xml_diff>